<commit_message>
merged no transmitters controller into a ui state view instead - and removed controller
</commit_message>
<xml_diff>
--- a/i18n/sheet.xlsx
+++ b/i18n/sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="22823"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="22904"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ehealthtrifork-my.sharepoint.com/personal/asg_dawnhealth_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1306" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{60A27A9B-E8F9-4E4C-890C-9200952112AA}"/>
+  <xr:revisionPtr revIDLastSave="1323" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{4CEB9BDA-EA37-4FC5-B0B5-0D790A48F3EB}"/>
   <bookViews>
-    <workbookView xWindow="60840" yWindow="2260" windowWidth="37540" windowHeight="25260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="60840" yWindow="2260" windowWidth="37540" windowHeight="25260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="guidelines (IFU)" sheetId="3" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1431" uniqueCount="638">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="643">
   <si>
     <t>English</t>
   </si>
@@ -1620,6 +1620,12 @@
     <t>Guides</t>
   </si>
   <si>
+    <t>menu_transmitters</t>
+  </si>
+  <si>
+    <t>Transmitters</t>
+  </si>
+  <si>
     <t>menu_settings</t>
   </si>
   <si>
@@ -1627,6 +1633,18 @@
   </si>
   <si>
     <t>Indstillinger</t>
+  </si>
+  <si>
+    <t>menu_subitem_profile</t>
+  </si>
+  <si>
+    <t>Profile</t>
+  </si>
+  <si>
+    <t>Profil</t>
+  </si>
+  <si>
+    <t>manu_subitem_profile</t>
   </si>
   <si>
     <t>menu_subItem_about</t>
@@ -1951,9 +1969,6 @@
   </si>
   <si>
     <t>transmitters_title</t>
-  </si>
-  <si>
-    <t>Transmitters</t>
   </si>
   <si>
     <t>transmitters_attached</t>
@@ -4601,7 +4616,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.42578125" style="2" customWidth="1"/>
@@ -6493,7 +6508,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="115" spans="1:8" ht="15.95">
+    <row r="115" spans="1:8">
       <c r="D115" s="2" t="s">
         <v>492</v>
       </c>
@@ -6504,7 +6519,7 @@
         <v>493</v>
       </c>
       <c r="G115" s="2" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="H115" s="2" t="s">
         <v>492</v>
@@ -6512,39 +6527,39 @@
     </row>
     <row r="116" spans="1:8" ht="15.95">
       <c r="D116" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="E116" s="2" t="s">
         <v>495</v>
       </c>
-      <c r="E116" s="2" t="s">
+      <c r="F116" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="G116" s="2" t="s">
         <v>496</v>
       </c>
-      <c r="F116" s="2" t="s">
-        <v>496</v>
-      </c>
-      <c r="G116" s="2" t="s">
+      <c r="H116" s="2" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8">
+      <c r="D117" s="2" t="s">
         <v>497</v>
       </c>
-      <c r="H116" s="2" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="117" spans="1:8" ht="15.95">
-      <c r="D117" s="2" t="s">
+      <c r="E117" s="2" t="s">
         <v>498</v>
       </c>
-      <c r="E117" s="2" t="s">
+      <c r="F117" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="G117" s="2" t="s">
         <v>499</v>
       </c>
-      <c r="F117" s="2" t="s">
-        <v>499</v>
-      </c>
-      <c r="G117" s="2" t="s">
+      <c r="H117" s="2" t="s">
         <v>500</v>
       </c>
-      <c r="H117" s="2" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="118" spans="1:8" ht="15.95">
+    </row>
+    <row r="118" spans="1:8">
       <c r="D118" s="2" t="s">
         <v>501</v>
       </c>
@@ -6595,96 +6610,96 @@
         <v>507</v>
       </c>
     </row>
-    <row r="121" spans="1:8">
-      <c r="A121" s="4"/>
-      <c r="B121" s="4"/>
-      <c r="C121" s="4"/>
-      <c r="D121" s="4"/>
-      <c r="E121" s="4"/>
-      <c r="F121" s="4"/>
-      <c r="G121" s="4"/>
-      <c r="H121" s="4"/>
+    <row r="121" spans="1:8" ht="15.95">
+      <c r="D121" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="E121" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="F121" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="G121" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="H121" s="2" t="s">
+        <v>510</v>
+      </c>
     </row>
     <row r="122" spans="1:8" ht="15.95">
       <c r="D122" s="2" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>511</v>
-      </c>
-      <c r="F122" s="8" t="s">
-        <v>511</v>
-      </c>
-      <c r="G122" s="8" t="s">
-        <v>512</v>
+        <v>514</v>
+      </c>
+      <c r="F122" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="G122" s="2" t="s">
+        <v>515</v>
       </c>
       <c r="H122" s="2" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="123" spans="1:8" ht="15.95">
-      <c r="D123" s="2" t="s">
         <v>513</v>
       </c>
-      <c r="E123" s="2" t="s">
-        <v>514</v>
-      </c>
-      <c r="F123" s="11" t="s">
-        <v>515</v>
-      </c>
-      <c r="G123" s="11" t="s">
-        <v>515</v>
-      </c>
-      <c r="H123" s="2" t="s">
-        <v>513</v>
-      </c>
+    </row>
+    <row r="123" spans="1:8">
+      <c r="A123" s="4"/>
+      <c r="B123" s="4"/>
+      <c r="C123" s="4"/>
+      <c r="D123" s="4"/>
+      <c r="E123" s="4"/>
+      <c r="F123" s="4"/>
+      <c r="G123" s="4"/>
+      <c r="H123" s="4"/>
     </row>
     <row r="124" spans="1:8" ht="15.95">
       <c r="D124" s="2" t="s">
-        <v>515</v>
-      </c>
-      <c r="E124" s="8" t="s">
         <v>516</v>
       </c>
+      <c r="E124" s="2" t="s">
+        <v>517</v>
+      </c>
       <c r="F124" s="8" t="s">
+        <v>517</v>
+      </c>
+      <c r="G124" s="8" t="s">
+        <v>518</v>
+      </c>
+      <c r="H124" s="2" t="s">
         <v>516</v>
-      </c>
-      <c r="G124" s="8" t="s">
-        <v>517</v>
-      </c>
-      <c r="H124" s="2" t="s">
-        <v>515</v>
       </c>
     </row>
     <row r="125" spans="1:8" ht="15.95">
       <c r="D125" s="2" t="s">
-        <v>518</v>
-      </c>
-      <c r="E125" s="8" t="s">
         <v>519</v>
       </c>
-      <c r="F125" s="8" t="s">
+      <c r="E125" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="F125" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="G125" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="H125" s="2" t="s">
         <v>519</v>
       </c>
-      <c r="G125" s="8" t="s">
-        <v>520</v>
-      </c>
-      <c r="H125" s="2" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="126" spans="1:8" ht="32.1">
+    </row>
+    <row r="126" spans="1:8" ht="15.95">
       <c r="D126" s="2" t="s">
         <v>521</v>
       </c>
-      <c r="E126" s="2" t="s">
+      <c r="E126" s="8" t="s">
         <v>522</v>
       </c>
-      <c r="F126" s="11" t="s">
-        <v>515</v>
-      </c>
-      <c r="G126" s="11" t="s">
-        <v>515</v>
+      <c r="F126" s="8" t="s">
+        <v>522</v>
+      </c>
+      <c r="G126" s="8" t="s">
+        <v>523</v>
       </c>
       <c r="H126" s="2" t="s">
         <v>521</v>
@@ -6692,384 +6707,384 @@
     </row>
     <row r="127" spans="1:8" ht="15.95">
       <c r="D127" s="2" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="E127" s="8" t="s">
-        <v>302</v>
+        <v>525</v>
       </c>
       <c r="F127" s="8" t="s">
-        <v>302</v>
+        <v>525</v>
       </c>
       <c r="G127" s="8" t="s">
-        <v>303</v>
+        <v>526</v>
       </c>
       <c r="H127" s="2" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="128" spans="1:8" ht="32.1">
       <c r="D128" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="E128" s="8" t="s">
+        <v>527</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="F128" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="G128" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="H128" s="2" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" ht="15.95">
+      <c r="D129" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="E129" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="F129" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="G129" s="8" t="s">
+        <v>303</v>
+      </c>
+      <c r="H129" s="2" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" ht="32.1">
+      <c r="D130" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="E130" s="8" t="s">
         <v>305</v>
       </c>
-      <c r="F128" s="8" t="s">
+      <c r="F130" s="8" t="s">
         <v>305</v>
       </c>
-      <c r="G128" s="8" t="s">
+      <c r="G130" s="8" t="s">
         <v>306</v>
       </c>
-      <c r="H128" s="2" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="129" spans="1:8" ht="15.95">
-      <c r="A129" s="4" t="s">
-        <v>525</v>
-      </c>
-      <c r="B129" s="4"/>
-      <c r="C129" s="4"/>
-      <c r="D129" s="4"/>
-      <c r="E129" s="4"/>
-      <c r="F129" s="4"/>
-      <c r="G129" s="4"/>
-      <c r="H129" s="4"/>
-    </row>
-    <row r="130" spans="1:8" ht="15.95">
-      <c r="D130" s="2" t="s">
-        <v>526</v>
-      </c>
-      <c r="E130" s="2" t="s">
-        <v>519</v>
-      </c>
-      <c r="F130" s="8" t="s">
-        <v>519</v>
-      </c>
-      <c r="G130" s="8" t="s">
-        <v>520</v>
-      </c>
       <c r="H130" s="2" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
     </row>
     <row r="131" spans="1:8" ht="15.95">
-      <c r="D131" s="2" t="s">
-        <v>527</v>
-      </c>
-      <c r="E131" s="2" t="s">
-        <v>528</v>
-      </c>
-      <c r="F131" s="8" t="s">
-        <v>528</v>
-      </c>
-      <c r="G131" s="8" t="s">
-        <v>529</v>
-      </c>
-      <c r="H131" s="2" t="s">
-        <v>527</v>
-      </c>
+      <c r="A131" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="B131" s="4"/>
+      <c r="C131" s="4"/>
+      <c r="D131" s="4"/>
+      <c r="E131" s="4"/>
+      <c r="F131" s="4"/>
+      <c r="G131" s="4"/>
+      <c r="H131" s="4"/>
     </row>
     <row r="132" spans="1:8" ht="15.95">
       <c r="D132" s="2" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="E132" s="2" t="s">
-        <v>516</v>
+        <v>525</v>
       </c>
       <c r="F132" s="8" t="s">
-        <v>516</v>
+        <v>525</v>
       </c>
       <c r="G132" s="8" t="s">
-        <v>517</v>
+        <v>526</v>
       </c>
       <c r="H132" s="2" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="133" spans="1:8">
-      <c r="A133" s="4"/>
-      <c r="B133" s="4"/>
-      <c r="C133" s="4"/>
-      <c r="D133" s="4"/>
-      <c r="E133" s="4"/>
-      <c r="F133" s="4"/>
-      <c r="G133" s="4"/>
-      <c r="H133" s="4"/>
-    </row>
-    <row r="134" spans="1:8" s="8" customFormat="1" ht="15.95">
-      <c r="D134" s="8" t="s">
-        <v>531</v>
-      </c>
-      <c r="E134" s="8" t="s">
         <v>532</v>
       </c>
+    </row>
+    <row r="133" spans="1:8" ht="15.95">
+      <c r="D133" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="E133" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="F133" s="8" t="s">
+        <v>534</v>
+      </c>
+      <c r="G133" s="8" t="s">
+        <v>535</v>
+      </c>
+      <c r="H133" s="2" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8" ht="15.95">
+      <c r="D134" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>522</v>
+      </c>
       <c r="F134" s="8" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="G134" s="8" t="s">
-        <v>532</v>
-      </c>
-      <c r="H134" s="8" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="135" spans="1:8" s="8" customFormat="1" ht="15.95">
-      <c r="D135" s="8" t="s">
-        <v>533</v>
-      </c>
-      <c r="E135" s="8" t="s">
-        <v>534</v>
-      </c>
-      <c r="F135" s="8" t="s">
-        <v>534</v>
-      </c>
-      <c r="G135" s="8" t="s">
-        <v>534</v>
-      </c>
-      <c r="H135" s="8" t="s">
-        <v>534</v>
-      </c>
+        <v>523</v>
+      </c>
+      <c r="H134" s="2" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8">
+      <c r="A135" s="4"/>
+      <c r="B135" s="4"/>
+      <c r="C135" s="4"/>
+      <c r="D135" s="4"/>
+      <c r="E135" s="4"/>
+      <c r="F135" s="4"/>
+      <c r="G135" s="4"/>
+      <c r="H135" s="4"/>
     </row>
     <row r="136" spans="1:8" s="8" customFormat="1" ht="15.95">
       <c r="D136" s="8" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="E136" s="8" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="F136" s="8" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="G136" s="8" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="H136" s="8" t="s">
-        <v>536</v>
-      </c>
-    </row>
-    <row r="137" spans="1:8" ht="15.95">
-      <c r="A137" s="4" t="s">
-        <v>537</v>
-      </c>
-      <c r="B137" s="4"/>
-      <c r="C137" s="4"/>
-      <c r="D137" s="4"/>
-      <c r="E137" s="4"/>
-      <c r="F137" s="4"/>
-      <c r="G137" s="4"/>
-      <c r="H137" s="4"/>
-    </row>
-    <row r="138" spans="1:8" ht="15.95">
-      <c r="D138" s="2" t="s">
         <v>538</v>
       </c>
-      <c r="E138" s="2" t="s">
-        <v>493</v>
-      </c>
-      <c r="F138" s="2" t="s">
-        <v>493</v>
-      </c>
-      <c r="G138" s="2" t="s">
-        <v>494</v>
-      </c>
-      <c r="H138" s="2" t="s">
+    </row>
+    <row r="137" spans="1:8" s="8" customFormat="1" ht="15.95">
+      <c r="D137" s="8" t="s">
         <v>539</v>
       </c>
+      <c r="E137" s="8" t="s">
+        <v>540</v>
+      </c>
+      <c r="F137" s="8" t="s">
+        <v>540</v>
+      </c>
+      <c r="G137" s="8" t="s">
+        <v>540</v>
+      </c>
+      <c r="H137" s="8" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" s="8" customFormat="1" ht="15.95">
+      <c r="D138" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="E138" s="8" t="s">
+        <v>542</v>
+      </c>
+      <c r="F138" s="8" t="s">
+        <v>542</v>
+      </c>
+      <c r="G138" s="8" t="s">
+        <v>542</v>
+      </c>
+      <c r="H138" s="8" t="s">
+        <v>542</v>
+      </c>
     </row>
     <row r="139" spans="1:8" ht="15.95">
-      <c r="D139" s="2" t="s">
-        <v>540</v>
-      </c>
-      <c r="E139" s="2" t="s">
-        <v>541</v>
-      </c>
-      <c r="F139" s="2" t="s">
-        <v>541</v>
-      </c>
-      <c r="G139" s="2" t="s">
-        <v>542</v>
-      </c>
-      <c r="H139" s="2" t="s">
-        <v>539</v>
-      </c>
+      <c r="A139" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="B139" s="4"/>
+      <c r="C139" s="4"/>
+      <c r="D139" s="4"/>
+      <c r="E139" s="4"/>
+      <c r="F139" s="4"/>
+      <c r="G139" s="4"/>
+      <c r="H139" s="4"/>
     </row>
     <row r="140" spans="1:8" ht="15.95">
       <c r="D140" s="2" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E140" s="2" t="s">
-        <v>539</v>
+        <v>495</v>
       </c>
       <c r="F140" s="2" t="s">
-        <v>539</v>
+        <v>495</v>
       </c>
       <c r="G140" s="2" t="s">
-        <v>539</v>
+        <v>496</v>
       </c>
       <c r="H140" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="141" spans="1:8" ht="15.95">
       <c r="D141" s="2" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="E141" s="2" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="F141" s="2" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="G141" s="2" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="H141" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="142" spans="1:8" ht="15.95">
       <c r="D142" s="2" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="E142" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="F142" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="G142" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H142" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="15.95">
       <c r="D143" s="2" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E143" s="2" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="F143" s="2" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="G143" s="2" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="H143" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="144" spans="1:8" ht="15.95">
       <c r="D144" s="2" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="E144" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="F144" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="G144" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H144" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="145" spans="1:8" ht="15.95">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="145" spans="4:8" ht="15.95">
       <c r="D145" s="2" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="E145" s="2" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="F145" s="2" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="G145" s="2" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="H145" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="146" spans="1:8" ht="15.95">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="146" spans="4:8" ht="15.95">
       <c r="D146" s="2" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="E146" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="F146" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="G146" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H146" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="147" spans="1:8" ht="15.95">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="147" spans="4:8" ht="15.95">
       <c r="D147" s="2" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="E147" s="2" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="F147" s="2" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="G147" s="2" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="H147" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="148" spans="1:8" ht="48">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="148" spans="4:8" ht="15.95">
       <c r="D148" s="2" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="E148" s="2" t="s">
-        <v>560</v>
+        <v>545</v>
       </c>
       <c r="F148" s="2" t="s">
-        <v>561</v>
+        <v>545</v>
       </c>
       <c r="G148" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="H148" s="2" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="149" spans="4:8" ht="15.95">
+      <c r="D149" s="2" t="s">
         <v>562</v>
       </c>
-      <c r="H148" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="149" spans="1:8" ht="15.95">
-      <c r="D149" s="2" t="s">
+      <c r="E149" s="2" t="s">
         <v>563</v>
       </c>
-      <c r="E149" s="2" t="s">
+      <c r="F149" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="G149" s="2" t="s">
         <v>564</v>
       </c>
-      <c r="F149" s="2" t="s">
-        <v>564</v>
-      </c>
-      <c r="G149" s="2" t="s">
+      <c r="H149" s="2" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="150" spans="4:8" ht="48">
+      <c r="D150" s="2" t="s">
         <v>565</v>
       </c>
-      <c r="H149" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="150" spans="1:8" ht="32.1">
-      <c r="D150" s="2" t="s">
+      <c r="E150" s="2" t="s">
         <v>566</v>
-      </c>
-      <c r="E150" s="2" t="s">
-        <v>567</v>
       </c>
       <c r="F150" s="2" t="s">
         <v>567</v>
@@ -7078,10 +7093,10 @@
         <v>568</v>
       </c>
       <c r="H150" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="151" spans="1:8" ht="15.95">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="151" spans="4:8" ht="15.95">
       <c r="D151" s="2" t="s">
         <v>569</v>
       </c>
@@ -7095,587 +7110,621 @@
         <v>571</v>
       </c>
       <c r="H151" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="152" spans="1:8" ht="15.95">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="152" spans="4:8" ht="32.1">
       <c r="D152" s="2" t="s">
         <v>572</v>
       </c>
       <c r="E152" s="2" t="s">
-        <v>539</v>
+        <v>573</v>
       </c>
       <c r="F152" s="2" t="s">
-        <v>539</v>
+        <v>573</v>
       </c>
       <c r="G152" s="2" t="s">
-        <v>539</v>
+        <v>574</v>
       </c>
       <c r="H152" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="153" spans="1:8" ht="15.95">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="153" spans="4:8" ht="15.95">
       <c r="D153" s="2" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="E153" s="2" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="F153" s="2" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="G153" s="2" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="H153" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="154" spans="1:8" ht="15.95">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="154" spans="4:8" ht="15.95">
       <c r="D154" s="2" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="E154" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="F154" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="G154" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H154" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="155" spans="1:8" ht="15.95">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="155" spans="4:8" ht="15.95">
       <c r="D155" s="2" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E155" s="2" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="F155" s="2" t="s">
-        <v>539</v>
+        <v>580</v>
       </c>
       <c r="G155" s="2" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="H155" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="156" spans="1:8" ht="48">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="156" spans="4:8" ht="15.95">
       <c r="D156" s="2" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E156" s="2" t="s">
-        <v>580</v>
+        <v>545</v>
       </c>
       <c r="F156" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="G156" s="2" t="s">
-        <v>580</v>
+        <v>545</v>
       </c>
       <c r="H156" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="157" spans="1:8" ht="15.95">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="157" spans="4:8" ht="15.95">
       <c r="D157" s="2" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E157" s="2" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="F157" s="2" t="s">
-        <v>582</v>
+        <v>545</v>
       </c>
       <c r="G157" s="2" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H157" s="2" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="158" spans="1:8" ht="15.95">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="158" spans="4:8" ht="48">
       <c r="D158" s="2" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="E158" s="2" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="F158" s="2" t="s">
-        <v>584</v>
+        <v>545</v>
       </c>
       <c r="G158" s="2" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="H158" s="2" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="159" spans="1:8" ht="15.95">
-      <c r="A159" s="4" t="s">
-        <v>585</v>
-      </c>
-      <c r="B159" s="4"/>
-      <c r="C159" s="4"/>
-      <c r="D159" s="4"/>
-      <c r="E159" s="4"/>
-      <c r="F159" s="4"/>
-      <c r="G159" s="4"/>
-      <c r="H159" s="4"/>
-    </row>
-    <row r="160" spans="1:8" ht="15.95">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="159" spans="4:8" ht="15.95">
+      <c r="D159" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="E159" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="F159" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="G159" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="H159" s="2" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="160" spans="4:8" ht="15.95">
       <c r="D160" s="2" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="E160" s="2" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="F160" s="2" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="G160" s="2" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="H160" s="2" t="s">
-        <v>539</v>
+        <v>590</v>
       </c>
     </row>
     <row r="161" spans="1:8" ht="15.95">
-      <c r="D161" s="2" t="s">
-        <v>589</v>
-      </c>
-      <c r="E161" s="2" t="s">
-        <v>539</v>
-      </c>
-      <c r="F161" s="2" t="s">
-        <v>539</v>
-      </c>
-      <c r="G161" s="2" t="s">
-        <v>539</v>
-      </c>
-      <c r="H161" s="2" t="s">
-        <v>539</v>
-      </c>
+      <c r="A161" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="B161" s="4"/>
+      <c r="C161" s="4"/>
+      <c r="D161" s="4"/>
+      <c r="E161" s="4"/>
+      <c r="F161" s="4"/>
+      <c r="G161" s="4"/>
+      <c r="H161" s="4"/>
     </row>
     <row r="162" spans="1:8" ht="15.95">
       <c r="D162" s="2" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="E162" s="2" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="F162" s="2" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="G162" s="2" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="H162" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="163" spans="1:8" ht="15.95">
       <c r="D163" s="2" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="E163" s="2" t="s">
-        <v>594</v>
+        <v>545</v>
       </c>
       <c r="F163" s="2" t="s">
-        <v>594</v>
+        <v>545</v>
       </c>
       <c r="G163" s="2" t="s">
-        <v>595</v>
+        <v>545</v>
       </c>
       <c r="H163" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="164" spans="1:8" ht="20.25" customHeight="1">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8" ht="15.95">
       <c r="D164" s="2" t="s">
         <v>596</v>
       </c>
       <c r="E164" s="2" t="s">
-        <v>539</v>
+        <v>597</v>
       </c>
       <c r="F164" s="2" t="s">
-        <v>539</v>
+        <v>597</v>
       </c>
       <c r="G164" s="2" t="s">
-        <v>539</v>
+        <v>598</v>
       </c>
       <c r="H164" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="165" spans="1:8" ht="15.95">
       <c r="D165" s="2" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="E165" s="2" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="F165" s="2" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="G165" s="2" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="H165" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="166" spans="1:8" ht="32.1">
-      <c r="A166" s="4" t="s">
-        <v>600</v>
-      </c>
-      <c r="B166" s="4"/>
-      <c r="C166" s="4"/>
-      <c r="D166" s="4"/>
-      <c r="E166" s="4"/>
-      <c r="F166" s="4"/>
-      <c r="G166" s="4"/>
-      <c r="H166" s="4"/>
+        <v>545</v>
+      </c>
+    </row>
+    <row r="166" spans="1:8" ht="20.25" customHeight="1">
+      <c r="D166" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="E166" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="F166" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="G166" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="H166" s="2" t="s">
+        <v>545</v>
+      </c>
     </row>
     <row r="167" spans="1:8" ht="15.95">
       <c r="D167" s="2" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="E167" s="2" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="F167" s="2" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="G167" s="2" t="s">
-        <v>539</v>
+        <v>605</v>
       </c>
       <c r="H167" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="168" spans="1:8" ht="15.95">
-      <c r="D168" s="2" t="s">
-        <v>603</v>
-      </c>
-      <c r="E168" s="2" t="s">
-        <v>604</v>
-      </c>
-      <c r="F168" s="2" t="s">
-        <v>604</v>
-      </c>
-      <c r="G168" s="2" t="s">
-        <v>539</v>
-      </c>
-      <c r="H168" s="2" t="s">
-        <v>539</v>
-      </c>
+        <v>545</v>
+      </c>
+    </row>
+    <row r="168" spans="1:8" ht="32.1">
+      <c r="A168" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="B168" s="4"/>
+      <c r="C168" s="4"/>
+      <c r="D168" s="4"/>
+      <c r="E168" s="4"/>
+      <c r="F168" s="4"/>
+      <c r="G168" s="4"/>
+      <c r="H168" s="4"/>
     </row>
     <row r="169" spans="1:8" ht="15.95">
       <c r="D169" s="2" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="E169" s="2" t="s">
-        <v>606</v>
+        <v>493</v>
       </c>
       <c r="F169" s="2" t="s">
-        <v>606</v>
+        <v>493</v>
       </c>
       <c r="G169" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H169" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="170" spans="1:8" ht="15.95">
       <c r="D170" s="2" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="E170" s="2" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="F170" s="2" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="G170" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H170" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="171" spans="1:8" ht="15.95">
       <c r="D171" s="2" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="E171" s="2" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="F171" s="2" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="G171" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H171" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="172" spans="1:8" ht="15.95">
       <c r="D172" s="2" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E172" s="2" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="F172" s="2" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="G172" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H172" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="173" spans="1:8" ht="15.95">
       <c r="D173" s="2" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="E173" s="2" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="F173" s="2" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="G173" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H173" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="174" spans="1:8" ht="15.95">
       <c r="D174" s="2" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E174" s="2" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="F174" s="2" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="G174" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H174" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="175" spans="1:8" ht="15.95">
       <c r="D175" s="2" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="E175" s="2" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="F175" s="2" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="G175" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H175" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="176" spans="1:8" ht="15.95">
       <c r="D176" s="2" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="E176" s="2" t="s">
-        <v>221</v>
+        <v>621</v>
       </c>
       <c r="F176" s="2" t="s">
-        <v>221</v>
+        <v>621</v>
       </c>
       <c r="G176" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H176" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="177" spans="1:8" ht="15.95">
       <c r="D177" s="2" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E177" s="2" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="F177" s="2" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="G177" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H177" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="179" spans="1:8" ht="32.1">
-      <c r="A179" s="4" t="s">
-        <v>622</v>
-      </c>
-      <c r="B179" s="4"/>
-      <c r="C179" s="4"/>
-      <c r="D179" s="4"/>
-      <c r="E179" s="4"/>
-      <c r="F179" s="4"/>
-      <c r="G179" s="4"/>
-      <c r="H179" s="4"/>
-    </row>
-    <row r="180" spans="1:8" ht="15.95">
-      <c r="D180" s="2" t="s">
-        <v>623</v>
-      </c>
-      <c r="E180" s="2" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="178" spans="1:8" ht="15.95">
+      <c r="D178" s="2" t="s">
         <v>624</v>
       </c>
-      <c r="F180" s="2" t="s">
-        <v>624</v>
-      </c>
-      <c r="G180" s="2" t="s">
-        <v>539</v>
-      </c>
-      <c r="H180" s="2" t="s">
-        <v>539</v>
+      <c r="E178" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="F178" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="G178" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="H178" s="2" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="179" spans="1:8" ht="15.95">
+      <c r="D179" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="E179" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="F179" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="G179" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="H179" s="2" t="s">
+        <v>545</v>
       </c>
     </row>
     <row r="181" spans="1:8" ht="32.1">
-      <c r="D181" s="2" t="s">
-        <v>625</v>
-      </c>
-      <c r="E181" s="2" t="s">
-        <v>626</v>
-      </c>
-      <c r="F181" s="2" t="s">
-        <v>626</v>
-      </c>
-      <c r="G181" s="2" t="s">
-        <v>539</v>
-      </c>
-      <c r="H181" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="182" spans="1:8" ht="32.1">
+      <c r="A181" s="4" t="s">
+        <v>627</v>
+      </c>
+      <c r="B181" s="4"/>
+      <c r="C181" s="4"/>
+      <c r="D181" s="4"/>
+      <c r="E181" s="4"/>
+      <c r="F181" s="4"/>
+      <c r="G181" s="4"/>
+      <c r="H181" s="4"/>
+    </row>
+    <row r="182" spans="1:8" ht="15.95">
       <c r="D182" s="2" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="E182" s="2" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="F182" s="2" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="G182" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H182" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="183" spans="1:8" ht="32.1">
       <c r="D183" s="2" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="E183" s="2" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="F183" s="2" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="G183" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H183" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="184" spans="1:8" ht="15.95">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="184" spans="1:8" ht="32.1">
       <c r="D184" s="2" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="E184" s="2" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="F184" s="2" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="G184" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H184" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="185" spans="1:8" ht="15.95">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="185" spans="1:8" ht="32.1">
       <c r="D185" s="2" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E185" s="2" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="F185" s="2" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="G185" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H185" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="186" spans="1:8" ht="32.1">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="186" spans="1:8" ht="15.95">
       <c r="D186" s="2" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="E186" s="2" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="F186" s="2" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="G186" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H186" s="2" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="187" spans="1:8" ht="32.1">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="187" spans="1:8" ht="15.95">
       <c r="D187" s="2" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="E187" s="2" t="s">
-        <v>539</v>
+        <v>639</v>
       </c>
       <c r="F187" s="2" t="s">
-        <v>539</v>
+        <v>639</v>
       </c>
       <c r="G187" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="H187" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
+      </c>
+    </row>
+    <row r="188" spans="1:8" ht="32.1">
+      <c r="D188" s="2" t="s">
+        <v>640</v>
+      </c>
+      <c r="E188" s="2" t="s">
+        <v>641</v>
+      </c>
+      <c r="F188" s="2" t="s">
+        <v>641</v>
+      </c>
+      <c r="G188" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="H188" s="2" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="189" spans="1:8" ht="32.1">
+      <c r="D189" s="2" t="s">
+        <v>642</v>
+      </c>
+      <c r="E189" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="F189" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="G189" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="H189" s="2" t="s">
+        <v>545</v>
       </c>
     </row>
   </sheetData>
@@ -7685,21 +7734,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001735E4C1AF81B044B42502EF65468AD3" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b06dd55da7e75ffac548536a232936d2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eadb902b-93b7-47a6-8130-18fdf8801a21" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="033944ded8f040f3b5ba86892713db09" ns2:_="">
     <xsd:import namespace="eadb902b-93b7-47a6-8130-18fdf8801a21"/>
@@ -7831,8 +7865,23 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FBDCD96-85A7-4ED3-BEE8-F34479CB9646}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B7D05CE-367F-41E4-8608-7D898D6C11DA}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7840,5 +7889,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B7D05CE-367F-41E4-8608-7D898D6C11DA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FBDCD96-85A7-4ED3-BEE8-F34479CB9646}"/>
 </file>
</xml_diff>